<commit_message>
terrestrial ecology finished + computer crash fixes + late commits
</commit_message>
<xml_diff>
--- a/Terrestrial Ecology/data.xlsx
+++ b/Terrestrial Ecology/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zojamancekpali/Desktop/KU Leuven/Terrestrial Ecology/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22370C83-2D5A-974D-ACEF-83B538E57B3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEB876C8-327F-D64A-9AA8-9AFB4724553B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29040" windowHeight="15720" firstSheet="10" activeTab="10" xr2:uid="{F5C02684-697E-4FBA-9D92-889A01CE8306}"/>
   </bookViews>
@@ -1549,22 +1549,22 @@
         <v>2.2999999999999998</v>
       </c>
       <c r="H1" s="22">
-        <v>3.1</v>
+        <v>11.1</v>
       </c>
       <c r="I1" s="22">
-        <v>3.2</v>
+        <v>11.2</v>
       </c>
       <c r="J1" s="22">
-        <v>3.3</v>
+        <v>11.3</v>
       </c>
       <c r="K1" s="22">
-        <v>4.0999999999999996</v>
+        <v>12.1</v>
       </c>
       <c r="L1" s="22">
-        <v>4.2</v>
+        <v>12.2</v>
       </c>
       <c r="M1" s="22">
-        <v>4.3</v>
+        <v>12.3</v>
       </c>
       <c r="N1" s="22">
         <v>5.0999999999999996</v>
@@ -13686,23 +13686,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="fd689c1b-2561-4a46-ae04-6449f963ff76" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100AF89B70DD9C08446A8443DF534F7285E" ma:contentTypeVersion="15" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="11ff1dea21826c897426cf024aa9a71a">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="04677cab-20cd-44d8-974c-14c664890eaa" xmlns:ns4="fd689c1b-2561-4a46-ae04-6449f963ff76" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="922e1b34d363eaf5969fb03f7bb01980" ns3:_="" ns4:_="">
     <xsd:import namespace="04677cab-20cd-44d8-974c-14c664890eaa"/>
@@ -13935,25 +13918,24 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{825FA823-3C51-4EA3-9A46-FE5B57DBFEBC}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="fd689c1b-2561-4a46-ae04-6449f963ff76" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{25A95B2E-F0AD-4F4C-96E0-84C63E13B21A}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="fd689c1b-2561-4a46-ae04-6449f963ff76"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1706160E-6C74-466C-916F-9A32C7FD56E0}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -13970,4 +13952,22 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{25A95B2E-F0AD-4F4C-96E0-84C63E13B21A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="fd689c1b-2561-4a46-ae04-6449f963ff76"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{825FA823-3C51-4EA3-9A46-FE5B57DBFEBC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>